<commit_message>
Caderno de pisos: produtos Portinari, rejunte, soleiras e corredor lateral
- P01 Santorini OFW NAT e P02 Santorini SGR HARD (dados do fabricante),
  coluna de rejunte (Corda, junta seca) e fichas dos porcelanatos
- Corredor lateral externo (P02 ou PI01) incluído no total geral
- Transições: soleira de mármore Itaúnas baguete 5 cm nas trocas de
  material e perfil metálico nos desníveis do mesmo material
- Removidas as referências e a fonte da medida do quadro de pisos

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KCYmec6LwRhJynzCnK2vyo
</commit_message>
<xml_diff>
--- a/caderno/quantitativos/QUANTITATIVOS PISOS E RODAPES - R00.xlsx
+++ b/caderno/quantitativos/QUANTITATIVOS PISOS E RODAPES - R00.xlsx
@@ -11,6 +11,8 @@
     <sheet name="Rodapés - memória" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Vãos" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Transições" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Soleiras" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Produtos" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -82,7 +84,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -126,6 +128,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -491,19 +494,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J30"/>
+  <dimension ref="A1:K30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
     <col width="42" customWidth="1" min="2" max="2"/>
-    <col width="38" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="90" customWidth="1" min="9" max="9"/>
-    <col width="40" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="90" customWidth="1" min="10" max="10"/>
+    <col width="30" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -539,20 +543,25 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Rejunte</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>Área adotada (m²)</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Área geometria DWG (m²)</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Fonte da medida</t>
-        </is>
-      </c>
       <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Memória da medida</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Controle</t>
         </is>
@@ -566,17 +575,18 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>PORCELANATO SANTORINI OFF WHITE (PADRÃO)</t>
+          <t>PORCELANATO SANTORINI OFW NAT</t>
         </is>
       </c>
       <c r="C2" s="2" t="n"/>
       <c r="D2" s="2" t="n"/>
       <c r="E2" s="2" t="n"/>
       <c r="F2" s="2" t="n"/>
-      <c r="G2" s="3" t="n"/>
-      <c r="H2" s="4" t="n"/>
-      <c r="I2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="3" t="n"/>
+      <c r="I2" s="4" t="n"/>
       <c r="J2" s="2" t="n"/>
+      <c r="K2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
@@ -591,36 +601,41 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>Porcelanato Santorini Off White (padrão)</t>
+          <t>Porcelanato Santorini OFW NAT</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>A CONFIRMAR ¹</t>
+          <t>Portinari</t>
         </is>
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t>A CONFIRMAR ¹</t>
+          <t>90 × 90 cm</t>
         </is>
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>A CONFIRMAR ¹</t>
-        </is>
-      </c>
-      <c r="G3" s="6" t="n">
+          <t>Natural (NAT)</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>Corda · junta seca</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="n">
         <v>28.7</v>
       </c>
-      <c r="H3" s="7" t="n">
+      <c r="I3" s="7" t="n">
         <v>28.525</v>
       </c>
-      <c r="I3" s="5" t="inlineStr">
+      <c r="J3" s="5" t="inlineStr">
         <is>
           <t>Rótulo DWG Prefeitura "SUÍTE MASTER A=28,70 m²" = valor informado; geometria DWG 16,28 + 12,25 = 28,53 (maior valor adotado)</t>
         </is>
       </c>
-      <c r="J3" s="5" t="inlineStr">
+      <c r="K3" s="5" t="inlineStr">
         <is>
           <t>Arquivo + Informado</t>
         </is>
@@ -639,36 +654,41 @@
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>Porcelanato Santorini Off White (padrão)</t>
+          <t>Porcelanato Santorini OFW NAT</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>A CONFIRMAR ¹</t>
+          <t>Portinari</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>A CONFIRMAR ¹</t>
+          <t>90 × 90 cm</t>
         </is>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>A CONFIRMAR ¹</t>
-        </is>
-      </c>
-      <c r="G4" s="6" t="n">
+          <t>Natural (NAT)</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>Corda · junta seca</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="n">
         <v>6.83</v>
       </c>
-      <c r="H4" s="7" t="n">
+      <c r="I4" s="7" t="n">
         <v>6.825</v>
       </c>
-      <c r="I4" s="5" t="inlineStr">
+      <c r="J4" s="5" t="inlineStr">
         <is>
           <t>Geometria DWG 1,95 × 3,50 = 6,83 (rótulo planta de piso 6,83); informado/Prefeitura 6,30 (maior valor adotado)</t>
         </is>
       </c>
-      <c r="J4" s="5" t="inlineStr">
+      <c r="K4" s="5" t="inlineStr">
         <is>
           <t>Arquivo</t>
         </is>
@@ -687,36 +707,41 @@
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Porcelanato Santorini Off White (padrão)</t>
+          <t>Porcelanato Santorini OFW NAT</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>A CONFIRMAR ¹</t>
+          <t>Portinari</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>A CONFIRMAR ¹</t>
+          <t>90 × 90 cm</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>A CONFIRMAR ¹</t>
-        </is>
-      </c>
-      <c r="G5" s="6" t="n">
+          <t>Natural (NAT)</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>Corda · junta seca</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="n">
         <v>12.3</v>
       </c>
-      <c r="H5" s="7" t="n">
+      <c r="I5" s="7" t="n">
         <v>12.3</v>
       </c>
-      <c r="I5" s="5" t="inlineStr">
+      <c r="J5" s="5" t="inlineStr">
         <is>
           <t>Geometria DWG 4,10 × 3,00 = rótulo 12,30 = informado</t>
         </is>
       </c>
-      <c r="J5" s="5" t="inlineStr">
+      <c r="K5" s="5" t="inlineStr">
         <is>
           <t>Arquivo + Informado</t>
         </is>
@@ -735,36 +760,41 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Porcelanato Santorini Off White (padrão)</t>
+          <t>Porcelanato Santorini OFW NAT</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>A CONFIRMAR ¹</t>
+          <t>Portinari</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>A CONFIRMAR ¹</t>
+          <t>90 × 90 cm</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>A CONFIRMAR ¹</t>
-        </is>
-      </c>
-      <c r="G6" s="6" t="n">
+          <t>Natural (NAT)</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>Corda · junta seca</t>
+        </is>
+      </c>
+      <c r="H6" s="6" t="n">
         <v>4.2</v>
       </c>
-      <c r="H6" s="7" t="n">
+      <c r="I6" s="7" t="n">
         <v>4.2</v>
       </c>
-      <c r="I6" s="5" t="inlineStr">
+      <c r="J6" s="5" t="inlineStr">
         <is>
           <t>Geometria DWG 2,80 × 1,50 = rótulo 4,20 = informado</t>
         </is>
       </c>
-      <c r="J6" s="5" t="inlineStr">
+      <c r="K6" s="5" t="inlineStr">
         <is>
           <t>Arquivo + Informado</t>
         </is>
@@ -783,36 +813,41 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Porcelanato Santorini Off White (padrão)</t>
+          <t>Porcelanato Santorini OFW NAT</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>A CONFIRMAR ¹</t>
+          <t>Portinari</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>A CONFIRMAR ¹</t>
+          <t>90 × 90 cm</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>A CONFIRMAR ¹</t>
-        </is>
-      </c>
-      <c r="G7" s="6" t="n">
+          <t>Natural (NAT)</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>Corda · junta seca</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="n">
         <v>12.3</v>
       </c>
-      <c r="H7" s="7" t="n">
+      <c r="I7" s="7" t="n">
         <v>12.3</v>
       </c>
-      <c r="I7" s="5" t="inlineStr">
+      <c r="J7" s="5" t="inlineStr">
         <is>
           <t>Geometria DWG 4,10 × 3,00 = rótulo 12,30 = informado</t>
         </is>
       </c>
-      <c r="J7" s="5" t="inlineStr">
+      <c r="K7" s="5" t="inlineStr">
         <is>
           <t>Arquivo + Informado</t>
         </is>
@@ -831,36 +866,41 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Porcelanato Santorini Off White (padrão)</t>
+          <t>Porcelanato Santorini OFW NAT</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>A CONFIRMAR ¹</t>
+          <t>Portinari</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>A CONFIRMAR ¹</t>
+          <t>90 × 90 cm</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>A CONFIRMAR ¹</t>
-        </is>
-      </c>
-      <c r="G8" s="6" t="n">
+          <t>Natural (NAT)</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>Corda · junta seca</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="n">
         <v>4.2</v>
       </c>
-      <c r="H8" s="7" t="n">
+      <c r="I8" s="7" t="n">
         <v>4.2</v>
       </c>
-      <c r="I8" s="5" t="inlineStr">
+      <c r="J8" s="5" t="inlineStr">
         <is>
           <t>Geometria DWG 2,80 × 1,50 = rótulo 4,20 = informado</t>
         </is>
       </c>
-      <c r="J8" s="5" t="inlineStr">
+      <c r="K8" s="5" t="inlineStr">
         <is>
           <t>Arquivo + Informado</t>
         </is>
@@ -879,36 +919,41 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Porcelanato Santorini Off White (padrão)</t>
+          <t>Porcelanato Santorini OFW NAT</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>A CONFIRMAR ¹</t>
+          <t>Portinari</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>A CONFIRMAR ¹</t>
+          <t>90 × 90 cm</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>A CONFIRMAR ¹</t>
-        </is>
-      </c>
-      <c r="G9" s="6" t="n">
+          <t>Natural (NAT)</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>Corda · junta seca</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="n">
         <v>7.26</v>
       </c>
-      <c r="H9" s="7" t="n">
+      <c r="I9" s="7" t="n">
         <v>7.26</v>
       </c>
-      <c r="I9" s="5" t="inlineStr">
+      <c r="J9" s="5" t="inlineStr">
         <is>
           <t>Geometria DWG 3,30 × 2,20 = rótulo 7,26 = informado</t>
         </is>
       </c>
-      <c r="J9" s="5" t="inlineStr">
+      <c r="K9" s="5" t="inlineStr">
         <is>
           <t>Arquivo + Informado</t>
         </is>
@@ -927,36 +972,41 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Porcelanato Santorini Off White (padrão)</t>
+          <t>Porcelanato Santorini OFW NAT</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>A CONFIRMAR ¹</t>
+          <t>Portinari</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>A CONFIRMAR ¹</t>
+          <t>90 × 90 cm</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>A CONFIRMAR ¹</t>
-        </is>
-      </c>
-      <c r="G10" s="6" t="n">
+          <t>Natural (NAT)</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>Corda · junta seca</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="n">
         <v>4.62</v>
       </c>
-      <c r="H10" s="7" t="n">
+      <c r="I10" s="7" t="n">
         <v>4.62</v>
       </c>
-      <c r="I10" s="5" t="inlineStr">
+      <c r="J10" s="5" t="inlineStr">
         <is>
           <t>Geometria DWG 3,30 × 1,40 = rótulo 4,62; informado/Prefeitura 4,27 (maior valor adotado)</t>
         </is>
       </c>
-      <c r="J10" s="5" t="inlineStr">
+      <c r="K10" s="5" t="inlineStr">
         <is>
           <t>Arquivo</t>
         </is>
@@ -975,36 +1025,41 @@
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Porcelanato Santorini Off White (padrão)</t>
+          <t>Porcelanato Santorini OFW NAT</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>A CONFIRMAR ¹</t>
+          <t>Portinari</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>A CONFIRMAR ¹</t>
+          <t>90 × 90 cm</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>A CONFIRMAR ¹</t>
-        </is>
-      </c>
-      <c r="G11" s="6" t="n">
+          <t>Natural (NAT)</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>Corda · junta seca</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="n">
         <v>12.85</v>
       </c>
-      <c r="H11" s="7" t="n">
+      <c r="I11" s="7" t="n">
         <v>12.285</v>
       </c>
-      <c r="I11" s="5" t="inlineStr">
+      <c r="J11" s="5" t="inlineStr">
         <is>
           <t>Rótulo DWG planta de piso/forro "CIRCULAÇÃO 12,85 m²"; geometria 1,20 × 8,40 + nicho 0,70 × 3,15 = 12,29; informado 10,08 (maior valor adotado)</t>
         </is>
       </c>
-      <c r="J11" s="5" t="inlineStr">
+      <c r="K11" s="5" t="inlineStr">
         <is>
           <t>Arquivo + Obra</t>
         </is>
@@ -1023,36 +1078,41 @@
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Porcelanato Santorini Off White (padrão)</t>
+          <t>Porcelanato Santorini OFW NAT</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>A CONFIRMAR ¹</t>
+          <t>Portinari</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>A CONFIRMAR ¹</t>
+          <t>90 × 90 cm</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>A CONFIRMAR ¹</t>
-        </is>
-      </c>
-      <c r="G12" s="6" t="n">
+          <t>Natural (NAT)</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>Corda · junta seca</t>
+        </is>
+      </c>
+      <c r="H12" s="6" t="n">
         <v>17.85</v>
       </c>
-      <c r="H12" s="7" t="n">
+      <c r="I12" s="7" t="n">
         <v>17.85</v>
       </c>
-      <c r="I12" s="5" t="inlineStr">
+      <c r="J12" s="5" t="inlineStr">
         <is>
           <t>Geometria DWG 4,25 × 4,20 = rótulo 17,85 = informado</t>
         </is>
       </c>
-      <c r="J12" s="5" t="inlineStr">
+      <c r="K12" s="5" t="inlineStr">
         <is>
           <t>Arquivo + Informado</t>
         </is>
@@ -1071,36 +1131,41 @@
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Porcelanato Santorini Off White (padrão)</t>
+          <t>Porcelanato Santorini OFW NAT</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>A CONFIRMAR ¹</t>
+          <t>Portinari</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>A CONFIRMAR ¹</t>
+          <t>90 × 90 cm</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>A CONFIRMAR ¹</t>
-        </is>
-      </c>
-      <c r="G13" s="6" t="n">
+          <t>Natural (NAT)</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>Corda · junta seca</t>
+        </is>
+      </c>
+      <c r="H13" s="6" t="n">
         <v>41.01</v>
       </c>
-      <c r="H13" s="7" t="n">
+      <c r="I13" s="7" t="n">
         <v>41.01</v>
       </c>
-      <c r="I13" s="5" t="inlineStr">
+      <c r="J13" s="5" t="inlineStr">
         <is>
           <t>Geometria DWG 5,25 × 8,00 − 1,65 × 0,60 = 41,01 = informado (Jantar 21,00 + Estar 20,01)</t>
         </is>
       </c>
-      <c r="J13" s="5" t="inlineStr">
+      <c r="K13" s="5" t="inlineStr">
         <is>
           <t>Arquivo + Informado</t>
         </is>
@@ -1119,36 +1184,41 @@
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>Porcelanato Santorini Off White (padrão)</t>
+          <t>Porcelanato Santorini OFW NAT</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>A CONFIRMAR ¹</t>
+          <t>Portinari</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>A CONFIRMAR ¹</t>
+          <t>90 × 90 cm</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>A CONFIRMAR ¹</t>
-        </is>
-      </c>
-      <c r="G14" s="6" t="n">
+          <t>Natural (NAT)</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>Corda · junta seca</t>
+        </is>
+      </c>
+      <c r="H14" s="6" t="n">
         <v>5.5</v>
       </c>
-      <c r="H14" s="7" t="n">
+      <c r="I14" s="7" t="n">
         <v>5.5</v>
       </c>
-      <c r="I14" s="5" t="inlineStr">
+      <c r="J14" s="5" t="inlineStr">
         <is>
           <t>Geometria DWG 2,75 × 2,00 = rótulo 5,50 = informado</t>
         </is>
       </c>
-      <c r="J14" s="5" t="inlineStr">
+      <c r="K14" s="5" t="inlineStr">
         <is>
           <t>Arquivo + Informado</t>
         </is>
@@ -1167,36 +1237,41 @@
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>Porcelanato Santorini Off White (padrão)</t>
+          <t>Porcelanato Santorini OFW NAT</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>A CONFIRMAR ¹</t>
+          <t>Portinari</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>A CONFIRMAR ¹</t>
+          <t>90 × 90 cm</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>A CONFIRMAR ¹</t>
-        </is>
-      </c>
-      <c r="G15" s="6" t="n">
+          <t>Natural (NAT)</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>Corda · junta seca</t>
+        </is>
+      </c>
+      <c r="H15" s="6" t="n">
         <v>2.4</v>
       </c>
-      <c r="H15" s="7" t="n">
+      <c r="I15" s="7" t="n">
         <v>2.4</v>
       </c>
-      <c r="I15" s="5" t="inlineStr">
+      <c r="J15" s="5" t="inlineStr">
         <is>
           <t>Geometria DWG 1,20 × 2,00 = rótulo 2,40 = informado</t>
         </is>
       </c>
-      <c r="J15" s="5" t="inlineStr">
+      <c r="K15" s="5" t="inlineStr">
         <is>
           <t>Arquivo + Informado</t>
         </is>
@@ -1215,36 +1290,41 @@
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>Porcelanato Santorini Off White (padrão)</t>
+          <t>Porcelanato Santorini OFW NAT</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>A CONFIRMAR ¹</t>
+          <t>Portinari</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>A CONFIRMAR ¹</t>
+          <t>90 × 90 cm</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>A CONFIRMAR ¹</t>
-        </is>
-      </c>
-      <c r="G16" s="6" t="n">
+          <t>Natural (NAT)</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>Corda · junta seca</t>
+        </is>
+      </c>
+      <c r="H16" s="6" t="n">
         <v>37.65</v>
       </c>
-      <c r="H16" s="7" t="n">
+      <c r="I16" s="7" t="n">
         <v>37.65</v>
       </c>
-      <c r="I16" s="5" t="inlineStr">
+      <c r="J16" s="5" t="inlineStr">
         <is>
           <t>Geometria DWG 7,40 × 5,10 − 0,15 × 0,60 = 37,65 (= rótulo planta de forro); informado/Prefeitura 36,97 (maior valor adotado)</t>
         </is>
       </c>
-      <c r="J16" s="5" t="inlineStr">
+      <c r="K16" s="5" t="inlineStr">
         <is>
           <t>Arquivo</t>
         </is>
@@ -1261,13 +1341,14 @@
       <c r="D17" s="8" t="inlineStr"/>
       <c r="E17" s="8" t="inlineStr"/>
       <c r="F17" s="8" t="inlineStr"/>
-      <c r="G17" s="9">
-        <f>SUM(G3:G16)</f>
+      <c r="G17" s="8" t="inlineStr"/>
+      <c r="H17" s="9">
+        <f>SUM(H3:H16)</f>
         <v/>
       </c>
-      <c r="H17" s="10" t="n"/>
-      <c r="I17" s="8" t="n"/>
+      <c r="I17" s="10" t="n"/>
       <c r="J17" s="8" t="n"/>
+      <c r="K17" s="8" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1277,17 +1358,18 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>PORCELANATO SANTORINI OFF WHITE HARD</t>
+          <t>PORCELANATO SANTORINI SGR HARD</t>
         </is>
       </c>
       <c r="C18" s="2" t="n"/>
       <c r="D18" s="2" t="n"/>
       <c r="E18" s="2" t="n"/>
       <c r="F18" s="2" t="n"/>
-      <c r="G18" s="3" t="n"/>
-      <c r="H18" s="4" t="n"/>
-      <c r="I18" s="2" t="n"/>
+      <c r="G18" s="2" t="n"/>
+      <c r="H18" s="3" t="n"/>
+      <c r="I18" s="4" t="n"/>
       <c r="J18" s="2" t="n"/>
+      <c r="K18" s="2" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
@@ -1302,7 +1384,7 @@
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>Porcelanato Santorini Off White HARD</t>
+          <t>Porcelanato Santorini SGR HARD</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
@@ -1317,21 +1399,26 @@
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>HARD (áreas externas)</t>
-        </is>
-      </c>
-      <c r="G19" s="6" t="n">
+          <t>HARD (antiderrapante)</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>Corda · junta seca</t>
+        </is>
+      </c>
+      <c r="H19" s="6" t="n">
         <v>18.32</v>
       </c>
-      <c r="H19" s="7" t="n">
+      <c r="I19" s="7" t="n">
         <v>18.315</v>
       </c>
-      <c r="I19" s="5" t="inlineStr">
+      <c r="J19" s="5" t="inlineStr">
         <is>
           <t>Contorno da hachura DWG 4,05 × 4,50 + 0,60 × 0,15 = 18,32; informado/Prefeitura 18,22 (maior valor adotado)</t>
         </is>
       </c>
-      <c r="J19" s="5" t="inlineStr">
+      <c r="K19" s="5" t="inlineStr">
         <is>
           <t>Arquivo</t>
         </is>
@@ -1350,7 +1437,7 @@
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>Porcelanato Santorini Off White HARD</t>
+          <t>Porcelanato Santorini SGR HARD</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
@@ -1365,21 +1452,26 @@
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>HARD (áreas externas)</t>
-        </is>
-      </c>
-      <c r="G20" s="6" t="n">
+          <t>HARD (antiderrapante)</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>Corda · junta seca</t>
+        </is>
+      </c>
+      <c r="H20" s="6" t="n">
         <v>77.69</v>
       </c>
-      <c r="H20" s="7" t="n">
+      <c r="I20" s="7" t="n">
         <v>77.688</v>
       </c>
-      <c r="I20" s="5" t="inlineStr">
+      <c r="J20" s="5" t="inlineStr">
         <is>
           <t>Hachura DWG 61,37 + giro P03 0,64 + faixas sob beiral 1,00 × 7,40 e 1,00 × 8,28 (beiral: DWG Prefeitura, "PROJEÇÃO DO BEIRAL")</t>
         </is>
       </c>
-      <c r="J20" s="5" t="inlineStr">
+      <c r="K20" s="5" t="inlineStr">
         <is>
           <t>Arquivo + Informado + Obra</t>
         </is>
@@ -1396,13 +1488,14 @@
       <c r="D21" s="8" t="inlineStr"/>
       <c r="E21" s="8" t="inlineStr"/>
       <c r="F21" s="8" t="inlineStr"/>
-      <c r="G21" s="9">
-        <f>SUM(G19:G20)</f>
+      <c r="G21" s="8" t="inlineStr"/>
+      <c r="H21" s="9">
+        <f>SUM(H19:H20)</f>
         <v/>
       </c>
-      <c r="H21" s="10" t="n"/>
-      <c r="I21" s="8" t="n"/>
+      <c r="I21" s="10" t="n"/>
       <c r="J21" s="8" t="n"/>
+      <c r="K21" s="8" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1419,10 +1512,11 @@
       <c r="D22" s="2" t="n"/>
       <c r="E22" s="2" t="n"/>
       <c r="F22" s="2" t="n"/>
-      <c r="G22" s="3" t="n"/>
-      <c r="H22" s="4" t="n"/>
-      <c r="I22" s="2" t="n"/>
+      <c r="G22" s="2" t="n"/>
+      <c r="H22" s="3" t="n"/>
+      <c r="I22" s="4" t="n"/>
       <c r="J22" s="2" t="n"/>
+      <c r="K22" s="2" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
@@ -1455,18 +1549,23 @@
           <t>A CONFIRMAR</t>
         </is>
       </c>
-      <c r="G23" s="6" t="n">
+      <c r="G23" s="5" t="inlineStr">
+        <is>
+          <t>A CONFIRMAR</t>
+        </is>
+      </c>
+      <c r="H23" s="6" t="n">
         <v>37</v>
       </c>
-      <c r="H23" s="7" t="n">
+      <c r="I23" s="7" t="n">
         <v>34.606</v>
       </c>
-      <c r="I23" s="5" t="inlineStr">
+      <c r="J23" s="5" t="inlineStr">
         <is>
           <t>Informado: 7,40 × 5,00 com margem; geometria DWG com borda curva = 34,61 (maior valor adotado)</t>
         </is>
       </c>
-      <c r="J23" s="5" t="inlineStr">
+      <c r="K23" s="5" t="inlineStr">
         <is>
           <t>Informado</t>
         </is>
@@ -1503,18 +1602,23 @@
           <t>A CONFIRMAR</t>
         </is>
       </c>
-      <c r="G24" s="6" t="n">
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>A CONFIRMAR</t>
+        </is>
+      </c>
+      <c r="H24" s="6" t="n">
         <v>15.03</v>
       </c>
-      <c r="H24" s="7" t="n">
+      <c r="I24" s="7" t="n">
         <v>15.027</v>
       </c>
-      <c r="I24" s="5" t="inlineStr">
+      <c r="J24" s="5" t="inlineStr">
         <is>
           <t>Hachura GRASS do DWG (pedra portuguesa) fora da rampa e das áreas verdes</t>
         </is>
       </c>
-      <c r="J24" s="5" t="inlineStr">
+      <c r="K24" s="5" t="inlineStr">
         <is>
           <t>Arquivo + Obra</t>
         </is>
@@ -1551,18 +1655,23 @@
           <t>A CONFIRMAR</t>
         </is>
       </c>
-      <c r="G25" s="6" t="n">
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>A CONFIRMAR</t>
+        </is>
+      </c>
+      <c r="H25" s="6" t="n">
         <v>98.06999999999999</v>
       </c>
-      <c r="H25" s="7" t="n">
+      <c r="I25" s="7" t="n">
         <v>98.068</v>
       </c>
-      <c r="I25" s="5" t="inlineStr">
+      <c r="J25" s="5" t="inlineStr">
         <is>
           <t>Geometria DWG: divisa frontal 40,32 m × faixas 1,25 + 1,10; término na Av. 3 não fechado no DWG</t>
         </is>
       </c>
-      <c r="J25" s="5" t="inlineStr">
+      <c r="K25" s="5" t="inlineStr">
         <is>
           <t>Arquivo + Obra</t>
         </is>
@@ -1579,13 +1688,14 @@
       <c r="D26" s="8" t="inlineStr"/>
       <c r="E26" s="8" t="inlineStr"/>
       <c r="F26" s="8" t="inlineStr"/>
-      <c r="G26" s="9">
-        <f>SUM(G23:G25)</f>
+      <c r="G26" s="8" t="inlineStr"/>
+      <c r="H26" s="9">
+        <f>SUM(H23:H25)</f>
         <v/>
       </c>
-      <c r="H26" s="10" t="n"/>
-      <c r="I26" s="8" t="n"/>
+      <c r="I26" s="10" t="n"/>
       <c r="J26" s="8" t="n"/>
+      <c r="K26" s="8" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1595,17 +1705,18 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>PISO NÃO DEFINIDO — A CONFIRMAR</t>
+          <t>A DEFINIR — P02 OU PI01 (INTERTRAVADO DRENANTE)</t>
         </is>
       </c>
       <c r="C27" s="2" t="n"/>
       <c r="D27" s="2" t="n"/>
       <c r="E27" s="2" t="n"/>
       <c r="F27" s="2" t="n"/>
-      <c r="G27" s="3" t="n"/>
-      <c r="H27" s="4" t="n"/>
-      <c r="I27" s="2" t="n"/>
+      <c r="G27" s="2" t="n"/>
+      <c r="H27" s="3" t="n"/>
+      <c r="I27" s="4" t="n"/>
       <c r="J27" s="2" t="n"/>
+      <c r="K27" s="2" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
@@ -1615,41 +1726,46 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>Corredor Lateral</t>
+          <t>Corredor Lateral Externo</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>Piso NÃO DEFINIDO</t>
+          <t>A DEFINIR: P02 ou PI01</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>A CONFIRMAR</t>
+          <t>Portinari / A CONFIRMAR</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>A CONFIRMAR</t>
+          <t>90 × 90 cm ou A CONFIRMAR</t>
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>A CONFIRMAR</t>
-        </is>
-      </c>
-      <c r="G28" s="6" t="n">
+          <t>HARD ou drenante</t>
+        </is>
+      </c>
+      <c r="G28" s="5" t="inlineStr">
+        <is>
+          <t>Corda ou A CONFIRMAR</t>
+        </is>
+      </c>
+      <c r="H28" s="6" t="n">
         <v>23.93</v>
       </c>
-      <c r="H28" s="7" t="n">
+      <c r="I28" s="7" t="n">
         <v>23.422</v>
       </c>
-      <c r="I28" s="5" t="inlineStr">
+      <c r="J28" s="5" t="inlineStr">
         <is>
           <t>Informado: 1,50 × 15,95 (aprox.); contorno da hachura DWG = 23,42 (maior valor adotado)</t>
         </is>
       </c>
-      <c r="J28" s="5" t="inlineStr">
+      <c r="K28" s="5" t="inlineStr">
         <is>
           <t>Informado + Obra</t>
         </is>
@@ -1666,32 +1782,34 @@
       <c r="D29" s="8" t="inlineStr"/>
       <c r="E29" s="8" t="inlineStr"/>
       <c r="F29" s="8" t="inlineStr"/>
-      <c r="G29" s="9">
-        <f>SUM(G28:G28)</f>
+      <c r="G29" s="8" t="inlineStr"/>
+      <c r="H29" s="9">
+        <f>SUM(H28:H28)</f>
         <v/>
       </c>
-      <c r="H29" s="10" t="n"/>
-      <c r="I29" s="8" t="n"/>
+      <c r="I29" s="10" t="n"/>
       <c r="J29" s="8" t="n"/>
+      <c r="K29" s="8" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="11" t="inlineStr"/>
       <c r="B30" s="11" t="inlineStr">
         <is>
-          <t>TOTAL GERAL ESPECIFICADO (P01 + P02 + PP01)</t>
+          <t>TOTAL GERAL (P01 + P02 + PP01 + a definir)</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr"/>
       <c r="D30" s="11" t="inlineStr"/>
       <c r="E30" s="11" t="inlineStr"/>
       <c r="F30" s="11" t="inlineStr"/>
-      <c r="G30" s="12">
-        <f>G17+G21+G26</f>
+      <c r="G30" s="11" t="inlineStr"/>
+      <c r="H30" s="12">
+        <f>H17+H21+H26+H29</f>
         <v/>
       </c>
-      <c r="H30" s="13" t="n"/>
-      <c r="I30" s="11" t="n"/>
+      <c r="I30" s="13" t="n"/>
       <c r="J30" s="11" t="n"/>
+      <c r="K30" s="11" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1779,7 +1897,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>RODAPÉ SANTORINI OFF WHITE PADRÃO — h = 8 cm</t>
+          <t>RODAPÉ PORCELANATO SANTORINI OFW NAT — h = 8 cm</t>
         </is>
       </c>
       <c r="C2" s="2" t="n"/>
@@ -6820,7 +6938,7 @@
       </c>
       <c r="B132" s="2" t="inlineStr">
         <is>
-          <t>RODAPÉ SANTORINI OFF WHITE HARD — h = 8 cm</t>
+          <t>RODAPÉ PORCELANATO SANTORINI SGR HARD — h = 8 cm</t>
         </is>
       </c>
       <c r="C132" s="2" t="n"/>
@@ -8335,7 +8453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -8343,6 +8461,7 @@
     <col width="50" customWidth="1" min="3" max="3"/>
     <col width="80" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8363,12 +8482,17 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Situação / decisão</t>
+          <t>Solução</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Controle</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Soleira mármore Itaúnas (m)</t>
         </is>
       </c>
     </row>
@@ -8385,18 +8509,21 @@
       </c>
       <c r="C2" s="14" t="inlineStr">
         <is>
-          <t>Garagem (P01) / Corredor Lateral (piso A CONFIRMAR)</t>
+          <t>Garagem (P01) / Corredor Lateral Externo (P02 ou PI01)</t>
         </is>
       </c>
       <c r="D2" s="14" t="inlineStr">
         <is>
-          <t>Encontro dependente da definição do piso do corredor lateral.</t>
+          <t>Soleira mármore Itaúnas, baguete 5 cm × comprimento do vão (0,80 m).</t>
         </is>
       </c>
       <c r="E2" s="14" t="inlineStr">
         <is>
-          <t>Decisão</t>
-        </is>
+          <t>Informado</t>
+        </is>
+      </c>
+      <c r="F2" s="14" t="n">
+        <v>0.8</v>
       </c>
     </row>
     <row r="3">
@@ -8412,18 +8539,21 @@
       </c>
       <c r="C3" s="14" t="inlineStr">
         <is>
-          <t>Lavanderia (P01) / Corredor Lateral (piso A CONFIRMAR)</t>
+          <t>Lavanderia (P01) / Corredor Lateral Externo (P02 ou PI01)</t>
         </is>
       </c>
       <c r="D3" s="14" t="inlineStr">
         <is>
-          <t>Porta de correr: trilho embutido no piso (caderno de esquadrias, notas 3 e 10).</t>
+          <t>Soleira mármore Itaúnas, baguete 5 cm × comprimento do vão (1,80 m). Compatibilizar com o trilho embutido (esquadrias, notas 3 e 10).</t>
         </is>
       </c>
       <c r="E3" s="14" t="inlineStr">
         <is>
-          <t>Decisão</t>
-        </is>
+          <t>Informado</t>
+        </is>
+      </c>
+      <c r="F3" s="14" t="n">
+        <v>1.8</v>
       </c>
     </row>
     <row r="4">
@@ -8444,13 +8574,16 @@
       </c>
       <c r="D4" s="14" t="inlineStr">
         <is>
-          <t>Troca padrão → HARD na linha da esquadria; trilho embutido (notas 3 e 10).</t>
+          <t>Soleira mármore Itaúnas, baguete 5 cm × comprimento do vão (3,00 m). Compatibilizar com o trilho embutido.</t>
         </is>
       </c>
       <c r="E4" s="14" t="inlineStr">
         <is>
-          <t>Arquivo</t>
-        </is>
+          <t>Informado</t>
+        </is>
+      </c>
+      <c r="F4" s="14" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="5">
@@ -8471,13 +8604,16 @@
       </c>
       <c r="D5" s="14" t="inlineStr">
         <is>
-          <t>Troca padrão → HARD na linha da esquadria; trilho embutido (notas 3 e 10).</t>
+          <t>Soleira mármore Itaúnas, baguete 5 cm × comprimento do vão (3,00 m). Compatibilizar com o trilho embutido.</t>
         </is>
       </c>
       <c r="E5" s="14" t="inlineStr">
         <is>
-          <t>Arquivo</t>
-        </is>
+          <t>Informado</t>
+        </is>
+      </c>
+      <c r="F5" s="14" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="6">
@@ -8498,13 +8634,16 @@
       </c>
       <c r="D6" s="14" t="inlineStr">
         <is>
-          <t>Troca padrão → HARD na linha da esquadria. Tipo de trilho da veneziana de correr A CONFIRMAR.</t>
+          <t>Soleira mármore Itaúnas, baguete 5 cm × comprimento do vão (2,70 m). Compatibilizar com o trilho da veneziana de correr.</t>
         </is>
       </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
-          <t>Decisão</t>
-        </is>
+          <t>Informado</t>
+        </is>
+      </c>
+      <c r="F6" s="14" t="n">
+        <v>2.7</v>
       </c>
     </row>
     <row r="7">
@@ -8525,13 +8664,16 @@
       </c>
       <c r="D7" s="14" t="inlineStr">
         <is>
-          <t>Troca padrão → HARD na linha da porta. Soleira A CONFIRMAR.</t>
+          <t>Soleira mármore Itaúnas, baguete 5 cm × comprimento do vão (0,80 m).</t>
         </is>
       </c>
       <c r="E7" s="14" t="inlineStr">
         <is>
-          <t>Decisão</t>
-        </is>
+          <t>Informado</t>
+        </is>
+      </c>
+      <c r="F7" s="14" t="n">
+        <v>0.8</v>
       </c>
     </row>
     <row r="8">
@@ -8552,13 +8694,16 @@
       </c>
       <c r="D8" s="14" t="inlineStr">
         <is>
-          <t>Troca HARD → pedra portuguesa na linha do portão. Arremate/soleira A CONFIRMAR.</t>
+          <t>Soleira mármore Itaúnas, baguete 5 cm × comprimento do vão (0,90 m).</t>
         </is>
       </c>
       <c r="E8" s="14" t="inlineStr">
         <is>
-          <t>Decisão</t>
-        </is>
+          <t>Informado</t>
+        </is>
+      </c>
+      <c r="F8" s="14" t="n">
+        <v>0.9</v>
       </c>
     </row>
     <row r="9">
@@ -8574,18 +8719,21 @@
       </c>
       <c r="C9" s="14" t="inlineStr">
         <is>
-          <t>Garagem (P01) / Rampa (PP01)</t>
+          <t>Garagem (P01) / Rampa (PP01) — frente aberta</t>
         </is>
       </c>
       <c r="D9" s="14" t="inlineStr">
         <is>
-          <t>Frente aberta da garagem (7,40 m, linha y = 15,036). Arremate/junta A CONFIRMAR.</t>
+          <t>Soleira mármore Itaúnas, baguete 5 cm × comprimento do vão (7,40 m, linha y = 15,036).</t>
         </is>
       </c>
       <c r="E9" s="14" t="inlineStr">
         <is>
-          <t>Decisão</t>
-        </is>
+          <t>Informado</t>
+        </is>
+      </c>
+      <c r="F9" s="14" t="n">
+        <v>7.4</v>
       </c>
     </row>
     <row r="10">
@@ -8601,18 +8749,21 @@
       </c>
       <c r="C10" s="14" t="inlineStr">
         <is>
-          <t>Garagem (P01) / Acesso externo (PP01) e área verde</t>
+          <t>Garagem (P01) / Acesso externo (PP01) — lateral aberta</t>
         </is>
       </c>
       <c r="D10" s="14" t="inlineStr">
         <is>
-          <t>Lateral aberta da garagem (4,50 m). Arremate A CONFIRMAR.</t>
+          <t>Soleira mármore Itaúnas, baguete 5 cm × comprimento do vão (4,50 m).</t>
         </is>
       </c>
       <c r="E10" s="14" t="inlineStr">
         <is>
-          <t>Decisão</t>
-        </is>
+          <t>Informado</t>
+        </is>
+      </c>
+      <c r="F10" s="14" t="n">
+        <v>4.5</v>
       </c>
     </row>
     <row r="11">
@@ -8633,14 +8784,15 @@
       </c>
       <c r="D11" s="14" t="inlineStr">
         <is>
-          <t>Mesmo acabamento: sem troca de material (limite de cobertura).</t>
+          <t>Mesmo material, sem desnível documentado: sem soleira. Havendo desnível: perfil metálico (mesmo material, somente com desnível).</t>
         </is>
       </c>
       <c r="E11" s="14" t="inlineStr">
         <is>
-          <t>Arquivo</t>
-        </is>
-      </c>
+          <t>Informado</t>
+        </is>
+      </c>
+      <c r="F11" s="14" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
@@ -8660,7 +8812,7 @@
       </c>
       <c r="D12" s="14" t="inlineStr">
         <is>
-          <t>Borda da piscina e acabamento de arremate não documentados: A CONFIRMAR.</t>
+          <t>Borda da piscina e arremate não documentados: A CONFIRMAR.</t>
         </is>
       </c>
       <c r="E12" s="14" t="inlineStr">
@@ -8668,6 +8820,7 @@
           <t>Decisão</t>
         </is>
       </c>
+      <c r="F12" s="14" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="14" t="inlineStr">
@@ -8695,6 +8848,7 @@
           <t>Decisão</t>
         </is>
       </c>
+      <c r="F13" s="14" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="14" t="inlineStr">
@@ -8714,14 +8868,15 @@
       </c>
       <c r="D14" s="14" t="inlineStr">
         <is>
-          <t>Mesmo material. Continuidade na divisa conforme execução: conferir em obra.</t>
+          <t>Mesmo material: sem soleira. Havendo desnível: perfil metálico (mesmo material, somente com desnível).</t>
         </is>
       </c>
       <c r="E14" s="14" t="inlineStr">
         <is>
-          <t>Obra</t>
-        </is>
-      </c>
+          <t>Informado</t>
+        </is>
+      </c>
+      <c r="F14" s="14" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="14" t="inlineStr">
@@ -8741,14 +8896,15 @@
       </c>
       <c r="D15" s="14" t="inlineStr">
         <is>
-          <t>Mesmo piso. P04 não está desenhada no DWG: posição do trilho A CONFIRMAR.</t>
+          <t>Mesmo material: sem soleira. Havendo desnível: perfil metálico (mesmo material, somente com desnível). Posição do trilho de P04 A CONFIRMAR.</t>
         </is>
       </c>
       <c r="E15" s="14" t="inlineStr">
         <is>
-          <t>Decisão</t>
-        </is>
-      </c>
+          <t>Informado</t>
+        </is>
+      </c>
+      <c r="F15" s="14" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="14" t="inlineStr">
@@ -8768,12 +8924,587 @@
       </c>
       <c r="D16" s="14" t="inlineStr">
         <is>
-          <t>Mesmo piso nos dois lados. Soleiras não documentadas: A CONFIRMAR se houver.</t>
+          <t>Mesmo material: sem soleira. Havendo desnível: perfil metálico (mesmo material, somente com desnível).</t>
         </is>
       </c>
       <c r="E16" s="14" t="inlineStr">
         <is>
-          <t>Decisão</t>
+          <t>Informado</t>
+        </is>
+      </c>
+      <c r="F16" s="14" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="55" customWidth="1" min="3" max="3"/>
+    <col width="48" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Transição</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Porta</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Encontro</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Soleira</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Comprimento (m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>T01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>P02</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Garagem (P01) / Corredor Lateral Externo (P02 ou PI01)</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Mármore Itaúnas, baguete 5 cm de profundidade</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>T02</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>P07</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Lavanderia (P01) / Corredor Lateral Externo (P02 ou PI01)</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Mármore Itaúnas, baguete 5 cm de profundidade</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>1.8</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>T03</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>P05</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Sala TV / Sala Jantar (P01) / Varanda Gourmet (P02)</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Mármore Itaúnas, baguete 5 cm de profundidade</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>T04</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>P05</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Sala TV / Sala Jantar (P01) / Deck (P02)</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Mármore Itaúnas, baguete 5 cm de profundidade</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>T05</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Quarto Casal (P01) / Deck (P02)</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Mármore Itaúnas, baguete 5 cm de profundidade</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>2.7</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>T06</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>P11</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Banheiro Externo (P01) / Deck (P02)</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Mármore Itaúnas, baguete 5 cm de profundidade</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>T07</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>P03</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Deck (P02) / Acesso externo (PP01)</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Mármore Itaúnas, baguete 5 cm de profundidade</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>T08</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Garagem (P01) / Rampa (PP01) — frente aberta</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Mármore Itaúnas, baguete 5 cm de profundidade</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>7.4</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>T09</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Garagem (P01) / Acesso externo (PP01) — lateral aberta</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Mármore Itaúnas, baguete 5 cm de profundidade</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="15" t="inlineStr"/>
+      <c r="B11" s="15" t="inlineStr"/>
+      <c r="C11" s="15" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="D11" s="15" t="inlineStr"/>
+      <c r="E11" s="15">
+        <f>SUM(E2:E10)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="110" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Código</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Especificação</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Descrição</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Porcelanato esmaltado Santorini OFW NAT (Off White), borda retificada</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Fabricação</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>900 × 900 mm · espessura 7,0 mm · monocalibre</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Embalagem</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>3 peças / 2,43 m² por caixa</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Uso</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>áreas internas (Cód. Portinari, variação V e classe de uso: A CONFIRMAR na ficha)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Junta</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>junta seca (fabricante)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Rejunte</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>cor Corda (sugerida pelo fabricante) · proposta: argamassa de rejuntamento tipo II, NBR 14992, em WCs, banheiros, cozinha e lavanderia; tipo I nas áreas secas</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>P02</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Descrição</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Porcelanato esmaltado Santorini SGR HARD (Stone Gray, cinza), cód. 62928, borda retificada</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>P02</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Fabricação</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>900 × 900 mm · espessura 8,0 mm · monocalibre</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>P02</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Embalagem</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>2 peças / 1,62 m² por caixa</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>P02</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Uso</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>USO 6 (residencial e comercial de tráfego intenso) · variação V3 · interno e externo</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>P02</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Junta</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>junta seca (fabricante)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>P02</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Rejunte</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>cor Corda (sugerida pelo fabricante) · proposta: argamassa de rejuntamento tipo II, NBR 14992 (área externa)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>P02 ou PI01</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Opção 1</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>P02 — Porcelanato Santorini SGR HARD (dados acima)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>P02 ou PI01</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Opção 2</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>PI01 — Piso intertravado drenante (lajota/bloquete de concreto): dimensões, espessura, cor e resistência A CONFIRMAR (anúncio não acessível)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr"/>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Fonte</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Links do fabricante informados pela arquitetura (Portinari). Conferir na ficha técnica vigente.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Caderno de pisos: folha de detalhes, vãos de porta e áreas do casal
- Folha 06/06 com detalhes ilustrativos: rodapé 8 cm, perfil metálico,
  soleira baguete em mármore Itaúnas e trilho embutido no piso
- Vão das portas marcado em branco na espessura da parede
- Áreas do Closet Casal e do Quarto Casal na planta de pisos
- Removida a transição Varanda Gourmet / Deck; transições renumeradas

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KCYmec6LwRhJynzCnK2vyo
</commit_message>
<xml_diff>
--- a/caderno/quantitativos/QUANTITATIVOS PISOS E RODAPES - R00.xlsx
+++ b/caderno/quantitativos/QUANTITATIVOS PISOS E RODAPES - R00.xlsx
@@ -8453,7 +8453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -8779,17 +8779,17 @@
       </c>
       <c r="C11" s="14" t="inlineStr">
         <is>
-          <t>Varanda Gourmet (P02) / Deck (P02)</t>
+          <t>Deck (P02) / Piscina</t>
         </is>
       </c>
       <c r="D11" s="14" t="inlineStr">
         <is>
-          <t>Mesmo material, sem desnível documentado: sem soleira. Havendo desnível: perfil metálico (mesmo material, somente com desnível).</t>
+          <t>Borda da piscina e arremate não documentados: A CONFIRMAR.</t>
         </is>
       </c>
       <c r="E11" s="14" t="inlineStr">
         <is>
-          <t>Informado</t>
+          <t>Decisão</t>
         </is>
       </c>
       <c r="F11" s="14" t="n"/>
@@ -8807,12 +8807,12 @@
       </c>
       <c r="C12" s="14" t="inlineStr">
         <is>
-          <t>Deck (P02) / Piscina</t>
+          <t>Deck (P02) e PP01 / áreas verdes</t>
         </is>
       </c>
       <c r="D12" s="14" t="inlineStr">
         <is>
-          <t>Borda da piscina e arremate não documentados: A CONFIRMAR.</t>
+          <t>Contenção/arremate entre piso e jardim não documentado: A CONFIRMAR.</t>
         </is>
       </c>
       <c r="E12" s="14" t="inlineStr">
@@ -8835,17 +8835,17 @@
       </c>
       <c r="C13" s="14" t="inlineStr">
         <is>
-          <t>Deck (P02) e PP01 / áreas verdes</t>
+          <t>Rampa (PP01) / Calçada (PP01) — divisa</t>
         </is>
       </c>
       <c r="D13" s="14" t="inlineStr">
         <is>
-          <t>Contenção/arremate entre piso e jardim não documentado: A CONFIRMAR.</t>
+          <t>Mesmo material: sem soleira. Havendo desnível: perfil metálico (mesmo material, somente com desnível).</t>
         </is>
       </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
-          <t>Decisão</t>
+          <t>Informado</t>
         </is>
       </c>
       <c r="F13" s="14" t="n"/>
@@ -8858,17 +8858,17 @@
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>P04</t>
         </is>
       </c>
       <c r="C14" s="14" t="inlineStr">
         <is>
-          <t>Rampa (PP01) / Calçada (PP01) — divisa</t>
+          <t>Cozinha (P01) / Sala TV / Sala Jantar (P01)</t>
         </is>
       </c>
       <c r="D14" s="14" t="inlineStr">
         <is>
-          <t>Mesmo material: sem soleira. Havendo desnível: perfil metálico (mesmo material, somente com desnível).</t>
+          <t>Mesmo material: sem soleira. Havendo desnível: perfil metálico (mesmo material, somente com desnível). Posição do trilho de P04 A CONFIRMAR.</t>
         </is>
       </c>
       <c r="E14" s="14" t="inlineStr">
@@ -8886,17 +8886,17 @@
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>P04</t>
+          <t>P06/P08/P09</t>
         </is>
       </c>
       <c r="C15" s="14" t="inlineStr">
         <is>
-          <t>Cozinha (P01) / Sala TV / Sala Jantar (P01)</t>
+          <t>Portas internas (P01 / P01)</t>
         </is>
       </c>
       <c r="D15" s="14" t="inlineStr">
         <is>
-          <t>Mesmo material: sem soleira. Havendo desnível: perfil metálico (mesmo material, somente com desnível). Posição do trilho de P04 A CONFIRMAR.</t>
+          <t>Mesmo material: sem soleira. Havendo desnível: perfil metálico (mesmo material, somente com desnível).</t>
         </is>
       </c>
       <c r="E15" s="14" t="inlineStr">
@@ -8905,34 +8905,6 @@
         </is>
       </c>
       <c r="F15" s="14" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="14" t="inlineStr">
-        <is>
-          <t>T15</t>
-        </is>
-      </c>
-      <c r="B16" s="14" t="inlineStr">
-        <is>
-          <t>P06/P08/P09</t>
-        </is>
-      </c>
-      <c r="C16" s="14" t="inlineStr">
-        <is>
-          <t>Portas internas (P01 / P01)</t>
-        </is>
-      </c>
-      <c r="D16" s="14" t="inlineStr">
-        <is>
-          <t>Mesmo material: sem soleira. Havendo desnível: perfil metálico (mesmo material, somente com desnível).</t>
-        </is>
-      </c>
-      <c r="E16" s="14" t="inlineStr">
-        <is>
-          <t>Informado</t>
-        </is>
-      </c>
-      <c r="F16" s="14" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Rodapé embutido na parede em toda a casa
Detalhe D1 redesenhado (face do rodapé alinhada ao acabamento da parede,
rebaixo no reboco); legendas, memória, planilha e pendências atualizadas.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KCYmec6LwRhJynzCnK2vyo
</commit_message>
<xml_diff>
--- a/caderno/quantitativos/QUANTITATIVOS PISOS E RODAPES - R00.xlsx
+++ b/caderno/quantitativos/QUANTITATIVOS PISOS E RODAPES - R00.xlsx
@@ -1897,7 +1897,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>RODAPÉ PORCELANATO SANTORINI OFW NAT — h = 8 cm</t>
+          <t>RODAPÉ EMBUTIDO — PORCELANATO SANTORINI OFW NAT — h = 8 cm</t>
         </is>
       </c>
       <c r="C2" s="2" t="n"/>
@@ -6938,7 +6938,7 @@
       </c>
       <c r="B132" s="2" t="inlineStr">
         <is>
-          <t>RODAPÉ PORCELANATO SANTORINI SGR HARD — h = 8 cm</t>
+          <t>RODAPÉ EMBUTIDO — PORCELANATO SANTORINI SGR HARD — h = 8 cm</t>
         </is>
       </c>
       <c r="C132" s="2" t="n"/>

</xml_diff>